<commit_message>
docs(tutorials): the dyke's seed sits over the slope face
The single starting circle moves from under the flat berm bench — a spot
nobody would seed — to (49, 45, Depth 15), centered over the slope face and
cutting mid-depth into the clays. Every sensible seed in that neighborhood
converges to the same 1.7443 trap basin, so the teaching numbers are
unchanged; inputs and solution figures regenerated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_james_bay.xlsx
+++ b/docs/lem/files/xslope_james_bay.xlsx
@@ -10943,10 +10943,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>86</v>
+        <v>49</v>
       </c>
       <c r="C3" s="3">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>

</xml_diff>